<commit_message>
Updates to all activity files
</commit_message>
<xml_diff>
--- a/_site/assets/downloads/1.3_Team_Information_Organisation_Review.xlsx
+++ b/_site/assets/downloads/1.3_Team_Information_Organisation_Review.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hpwqld.sharepoint.com/sites/CDSDCT/Shared Documents/Digital Capability Framework POW/3. AP Delivery/2.0 Digital Literacy/06 Project Documentation/Build/GitHub Downloadable Resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="18" documentId="11_FBEC22EE00B46E68AB2061AC2AF43B4535999938" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{91E16E99-7B15-419E-B9A0-A32F8D472200}"/>
+  <xr:revisionPtr revIDLastSave="19" documentId="11_FBEC22EE00B46E68AB2061AC2AF43B4535999938" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{12BAA6CF-CE90-41E2-BC4D-D2AD60DA5301}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -227,17 +227,12 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFBF9FC"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -284,38 +279,38 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -630,7 +625,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="34" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="6"/>
@@ -639,13 +634,13 @@
       <c r="E1" s="6"/>
     </row>
     <row r="2" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="8"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="1"/>
@@ -655,22 +650,22 @@
       <c r="E3" s="1"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
       <c r="B4" s="1"/>
-      <c r="C4" s="9" t="s">
+      <c r="C4" s="2" t="s">
         <v>3</v>
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A5" s="9" t="s">
+      <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B5" s="1"/>
-      <c r="C5" s="9" t="s">
+      <c r="C5" s="2" t="s">
         <v>5</v>
       </c>
       <c r="D5" s="1"/>
@@ -684,7 +679,7 @@
       <c r="E6" s="1"/>
     </row>
     <row r="7" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="10" t="s">
+      <c r="A7" s="5" t="s">
         <v>6</v>
       </c>
       <c r="B7" s="6"/>
@@ -709,7 +704,7 @@
       <c r="E9" s="1"/>
     </row>
     <row r="10" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="10" t="s">
+      <c r="A10" s="5" t="s">
         <v>8</v>
       </c>
       <c r="B10" s="6"/>
@@ -734,7 +729,7 @@
       <c r="E12" s="1"/>
     </row>
     <row r="13" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="10" t="s">
+      <c r="A13" s="5" t="s">
         <v>10</v>
       </c>
       <c r="B13" s="6"/>
@@ -786,7 +781,7 @@
       <c r="E18" s="1"/>
     </row>
     <row r="19" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="10" t="s">
+      <c r="A19" s="5" t="s">
         <v>15</v>
       </c>
       <c r="B19" s="6"/>
@@ -795,125 +790,125 @@
       <c r="E19" s="6"/>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A20" s="11" t="s">
+      <c r="A20" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B20" s="11" t="s">
+      <c r="B20" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C20" s="11" t="s">
+      <c r="C20" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D20" s="11" t="s">
+      <c r="D20" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E20" s="11" t="s">
+      <c r="E20" s="3" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="12">
+      <c r="A21" s="10">
         <v>1</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="B21" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="C21" s="2"/>
-      <c r="D21" s="3" t="s">
+      <c r="C21" s="11"/>
+      <c r="D21" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="E21" s="2"/>
+      <c r="E21" s="11"/>
     </row>
     <row r="22" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="12">
+      <c r="A22" s="10">
         <v>2</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B22" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="C22" s="2"/>
-      <c r="D22" s="3" t="s">
+      <c r="C22" s="11"/>
+      <c r="D22" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="E22" s="2"/>
+      <c r="E22" s="11"/>
     </row>
     <row r="23" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="12">
+      <c r="A23" s="10">
         <v>3</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="B23" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="C23" s="2"/>
-      <c r="D23" s="3" t="s">
+      <c r="C23" s="11"/>
+      <c r="D23" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="E23" s="2"/>
+      <c r="E23" s="11"/>
     </row>
     <row r="24" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="12">
+      <c r="A24" s="10">
         <v>4</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="B24" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="C24" s="2"/>
-      <c r="D24" s="3" t="s">
+      <c r="C24" s="11"/>
+      <c r="D24" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="E24" s="2"/>
+      <c r="E24" s="11"/>
     </row>
     <row r="25" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="12">
+      <c r="A25" s="10">
         <v>5</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="B25" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="C25" s="2"/>
-      <c r="D25" s="3" t="s">
+      <c r="C25" s="11"/>
+      <c r="D25" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="E25" s="2"/>
+      <c r="E25" s="11"/>
     </row>
     <row r="26" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="12">
+      <c r="A26" s="10">
         <v>6</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="B26" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="C26" s="2"/>
-      <c r="D26" s="3" t="s">
+      <c r="C26" s="11"/>
+      <c r="D26" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="E26" s="2"/>
+      <c r="E26" s="11"/>
     </row>
     <row r="27" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="12">
+      <c r="A27" s="10">
         <v>7</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="B27" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="C27" s="2"/>
-      <c r="D27" s="3" t="s">
+      <c r="C27" s="11"/>
+      <c r="D27" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="E27" s="2"/>
+      <c r="E27" s="11"/>
     </row>
     <row r="28" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="12">
+      <c r="A28" s="10">
         <v>8</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="B28" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="C28" s="2"/>
-      <c r="D28" s="3" t="s">
+      <c r="C28" s="11"/>
+      <c r="D28" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="E28" s="2"/>
+      <c r="E28" s="11"/>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" s="1"/>
@@ -923,7 +918,7 @@
       <c r="E29" s="1"/>
     </row>
     <row r="30" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="10" t="s">
+      <c r="A30" s="5" t="s">
         <v>30</v>
       </c>
       <c r="B30" s="6"/>
@@ -966,7 +961,7 @@
       <c r="E34" s="1"/>
     </row>
     <row r="35" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="10" t="s">
+      <c r="A35" s="5" t="s">
         <v>34</v>
       </c>
       <c r="B35" s="6"/>
@@ -1000,7 +995,7 @@
       <c r="E38" s="1"/>
     </row>
     <row r="39" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="10" t="s">
+      <c r="A39" s="5" t="s">
         <v>37</v>
       </c>
       <c r="B39" s="6"/>
@@ -1049,7 +1044,7 @@
       <c r="E43" s="1"/>
     </row>
     <row r="44" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="10" t="s">
+      <c r="A44" s="5" t="s">
         <v>42</v>
       </c>
       <c r="B44" s="6"/>
@@ -1087,6 +1082,25 @@
   </sheetData>
   <autoFilter ref="A20:E28" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="35">
+    <mergeCell ref="A15:E15"/>
+    <mergeCell ref="C31:E31"/>
+    <mergeCell ref="A45:B45"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="C46:E46"/>
+    <mergeCell ref="A40:D40"/>
+    <mergeCell ref="C36:E36"/>
+    <mergeCell ref="A42:D42"/>
+    <mergeCell ref="A16:E16"/>
+    <mergeCell ref="A7:E7"/>
+    <mergeCell ref="A37:B37"/>
+    <mergeCell ref="A46:B46"/>
+    <mergeCell ref="C32:E32"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="C37:E37"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="A30:E30"/>
+    <mergeCell ref="A39:E39"/>
     <mergeCell ref="A47:B47"/>
     <mergeCell ref="A32:B32"/>
     <mergeCell ref="A41:D41"/>
@@ -1103,25 +1117,6 @@
     <mergeCell ref="A31:B31"/>
     <mergeCell ref="C47:E47"/>
     <mergeCell ref="A11:E11"/>
-    <mergeCell ref="A36:B36"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="C46:E46"/>
-    <mergeCell ref="A40:D40"/>
-    <mergeCell ref="C36:E36"/>
-    <mergeCell ref="A42:D42"/>
-    <mergeCell ref="A16:E16"/>
-    <mergeCell ref="A7:E7"/>
-    <mergeCell ref="A37:B37"/>
-    <mergeCell ref="A46:B46"/>
-    <mergeCell ref="C32:E32"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="C37:E37"/>
-    <mergeCell ref="A33:B33"/>
-    <mergeCell ref="A30:E30"/>
-    <mergeCell ref="A39:E39"/>
-    <mergeCell ref="A15:E15"/>
-    <mergeCell ref="C31:E31"/>
-    <mergeCell ref="A45:B45"/>
   </mergeCells>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape"/>
@@ -1143,15 +1138,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010066AE4C6A13B8E141A8E674DFA32CA6F2" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="5761630454da6c2d94458fc443ef2e29">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="25084aa5-12fd-4011-b528-cc6f0e62d12b" xmlns:ns3="3d81d758-da71-42ef-a10b-ca28e43b4f75" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="f7e2faffedb6149b0744f7bb7ad460f5" ns2:_="" ns3:_="">
     <xsd:import namespace="25084aa5-12fd-4011-b528-cc6f0e62d12b"/>
@@ -1386,6 +1372,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{973279F3-AD17-4FE2-9E51-D1CDEE30A2E7}">
   <ds:schemaRefs>
@@ -1398,14 +1393,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBE0916D-E0A4-4440-8ABB-A3BF3B946789}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3648ADBE-820F-4C4F-9445-B7054C7ADEA9}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1422,4 +1409,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBE0916D-E0A4-4440-8ABB-A3BF3B946789}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>